<commit_message>
Updated folder name and added file
</commit_message>
<xml_diff>
--- a/Estimates/BakeWBS.xlsx
+++ b/Estimates/BakeWBS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhishek.gaonkar\Downloads\Proposals\Momentive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhishek.gaonkar\Downloads\Proposals\Momentive\Estimates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1089DBA-D754-4E44-9D0B-2E1EB53E6C34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB9843E2-EE4A-462D-81A9-2FA592F8E71F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{5E186C5E-8EC3-4EDF-94DE-9500F4BA815C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="107">
   <si>
     <t xml:space="preserve">ID </t>
   </si>
@@ -334,6 +334,18 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>weeks</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>hours</t>
   </si>
 </sst>
 </file>
@@ -853,7 +865,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D79ED0E2-FD05-4D29-9225-20B8A827F914}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr defaultColWidth="19.453125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.1796875" style="2" bestFit="1" customWidth="1"/>
@@ -2391,13 +2403,35 @@
         <f>SUM(C3:C76)</f>
         <v>2248</v>
       </c>
-      <c r="D78" s="2">
+      <c r="D78" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C79" s="2">
         <f>C78/8</f>
         <v>281</v>
       </c>
-      <c r="E78" s="2">
-        <f>D78/5</f>
+      <c r="D79" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C80" s="2">
+        <f>C79/5</f>
         <v>56.2</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="81" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C81" s="2">
+        <f>C80/4</f>
+        <v>14.05</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>